<commit_message>
feat: update student import functionality to use exact ages instead of age ranges
- Modified the student import template to include "Age" instead of "Age Range".
- Updated the parsing logic to handle exact ages, ensuring validation for ages between 0 and 120.
- Adjusted related tests to reflect changes in age handling and validation.
- Enhanced user interface messages to align with the new age input requirements.
- Implemented backend logic to map exact ages to corresponding age-range labels for consistency.
</commit_message>
<xml_diff>
--- a/apps/step-up/public/templates/student-import-template.xlsx
+++ b/apps/step-up/public/templates/student-import-template.xlsx
@@ -19,7 +19,7 @@
     <t>Gender</t>
   </si>
   <si>
-    <t>Age Range</t>
+    <t>Age</t>
   </si>
   <si>
     <t>Ada Lovelace</t>
@@ -31,7 +31,7 @@
     <t>Female</t>
   </si>
   <si>
-    <t>20-40</t>
+    <t>28</t>
   </si>
   <si>
     <t>Alan Turing</t>
@@ -43,7 +43,7 @@
     <t>Male</t>
   </si>
   <si>
-    <t>10-20</t>
+    <t>16</t>
   </si>
 </sst>
 </file>

</xml_diff>